<commit_message>
Update landing hero and Halloumi Doner photos
</commit_message>
<xml_diff>
--- a/outputs/menu/menu.xlsx
+++ b/outputs/menu/menu.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R09150d3ed7e049f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Rdc09b83e6aeb439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="R08226921d4824179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="Rd3137d5f5c364e8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R28dc1d1978c740a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Ra8fab4c7307d4ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rb0cf7503ef54493e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="Rcf0e91b949d24b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8ff71d14f9134cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R4731aee7e3fe47f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="R503d42d88dab4f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="Rac3e4a23f3954161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="Rc84e72577c9d4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="R15bf031a91694294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rae656ba106fc4259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R00b3611862124588"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77af4c450e504669"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05da9b5436634d7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -698,7 +698,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T3" s="1" t="str">
-        <x:v>assets/images/Items/Halloumi–Kana Döner Ateria.jpg</x:v>
+        <x:v>assets/images/Items/Halloumi Kana Doner.png|assets/images/Items/Halloumi–Kana Döner Ateria.jpg</x:v>
       </x:c>
       <x:c r="U3" s="1" t="str"/>
       <x:c r="V3" s="1" t="str"/>
@@ -2804,7 +2804,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70cbc6bbb53249a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30f3a0ef412343e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3025,7 +3025,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9df22786df54fd5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9c62ec1fa464c02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3105,7 +3105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43947aa750a94cd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e9c1fbfdbb4479"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3209,7 +3209,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63707299cd3c4fde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa0d0b9b3a24f06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3396,7 +3396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bfd040e0b564778"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38b8494359134266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3564,7 +3564,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R690778a40ac94f75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b6ca32984344964"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update branding donation message and Facebook link
</commit_message>
<xml_diff>
--- a/outputs/menu/menu.xlsx
+++ b/outputs/menu/menu.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8ff71d14f9134cce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R4731aee7e3fe47f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="R503d42d88dab4f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="Rac3e4a23f3954161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="Rc84e72577c9d4bf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="R15bf031a91694294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rae656ba106fc4259"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R00b3611862124588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1be02eb5c5d64c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R1505bfb6451d4986"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="R60a4a0bbf15140c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="Rad3c70873205447f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="Rfe33896c63014205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="R2370a22034a44678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="R3c8bf3992bc5489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R88f49648841448f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05da9b5436634d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1639c43522ab4c4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2804,7 +2804,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30f3a0ef412343e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f172bb4d2184b5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3025,7 +3025,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9c62ec1fa464c02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c5f167f52f14201"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3105,7 +3105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e9c1fbfdbb4479"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4054ef8c68ab42ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3209,7 +3209,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa0d0b9b3a24f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae04f3d0d59d4bed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3396,7 +3396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38b8494359134266"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R679d67affa074d18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3546,7 +3546,7 @@
         <x:v>https://instagram.com/spicedonor</x:v>
       </x:c>
       <x:c r="R2" s="1" t="str">
-        <x:v>https://facebook.com/spicedonor</x:v>
+        <x:v>https://fb.com/spicedoner</x:v>
       </x:c>
       <x:c r="S2" s="1" t="str">
         <x:v>https://tiktok.com/@spicedonor</x:v>
@@ -3564,7 +3564,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b6ca32984344964"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8deb99550e994236"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>